<commit_message>
Finalise session: state files updated, R3 assets removed
- whats-next.md: reflects current tool state and open decisions
- TO-DOS.md: added items #33-35 (caption on page, PDF export, R3 removal)
- R3.svg deleted (R3 variant removed from tool)
- Old Spread 1.pdf deleted (superseded)
- Spread 1 - test.xlsx updated

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/Template_Toddler/Spread 1 - test.xlsx
+++ b/assets/Template_Toddler/Spread 1 - test.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/69cce5cfa03fbf09/Documents/AEVIA/Printing/Build backend tool/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evgmy\aevia-test\assets\Template_Toddler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{90B9181B-12D5-491C-96B5-EC5C8344026B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8B0BA50-C586-4DE3-BEED-7425A165BF0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4CBB4F2B-0595-4806-B8F1-C071DA4BF2B6}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sizing new'!$B$4:$M$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sizing new'!$B$4:$O$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="30">
   <si>
     <t>cells to fill</t>
   </si>
@@ -112,6 +112,27 @@
   </si>
   <si>
     <t>R3</t>
+  </si>
+  <si>
+    <t>captions_allowed</t>
+  </si>
+  <si>
+    <t>captions_position</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>below</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>above / below</t>
+  </si>
+  <si>
+    <t>yes / no</t>
   </si>
 </sst>
 </file>
@@ -569,38 +590,44 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB3C76F7-BD52-48B3-B788-24276A9CAB57}">
-  <dimension ref="B1:P12"/>
+  <dimension ref="B1:R12"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.109375" customWidth="1"/>
     <col min="2" max="8" width="17.109375" customWidth="1"/>
-    <col min="9" max="13" width="23.109375" customWidth="1"/>
-    <col min="14" max="16" width="8.77734375" style="2"/>
+    <col min="9" max="15" width="23.109375" customWidth="1"/>
+    <col min="16" max="18" width="8.77734375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
     </row>
-    <row r="3" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E3" s="4" t="s">
         <v>2</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="L3" t="s">
+        <v>29</v>
+      </c>
+      <c r="M3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="6" t="s">
         <v>4</v>
       </c>
@@ -632,16 +659,22 @@
         <v>13</v>
       </c>
       <c r="L4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="N4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="M4" s="7" t="s">
+      <c r="O4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
       <c r="P4" s="8"/>
-    </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="Q4" s="8"/>
+      <c r="R4" s="8"/>
+    </row>
+    <row r="5" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>1</v>
       </c>
@@ -675,13 +708,19 @@
         <v>horizontal</v>
       </c>
       <c r="L5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>1</v>
       </c>
@@ -715,13 +754,19 @@
         <v>vertical</v>
       </c>
       <c r="L6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="N6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="O6" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>1</v>
       </c>
@@ -755,13 +800,17 @@
         <v>horizontal</v>
       </c>
       <c r="L7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="O7" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>1</v>
       </c>
@@ -795,13 +844,17 @@
         <v>horizontal</v>
       </c>
       <c r="L8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="M8" s="1" t="s">
+      <c r="O8" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>1</v>
       </c>
@@ -835,13 +888,17 @@
         <v>vertical</v>
       </c>
       <c r="L9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="M9" s="1" t="s">
+      <c r="O9" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>1</v>
       </c>
@@ -875,13 +932,17 @@
         <v>vertical</v>
       </c>
       <c r="L10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="M10" s="1" t="s">
+      <c r="O10" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>1</v>
       </c>
@@ -915,13 +976,17 @@
         <v>vertical</v>
       </c>
       <c r="L11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="M11" s="1" t="s">
+      <c r="O11" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>1</v>
       </c>
@@ -955,14 +1020,18 @@
         <v>horizontal</v>
       </c>
       <c r="L12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="M12" s="1" t="s">
+      <c r="O12" s="1" t="s">
         <v>18</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:M4" xr:uid="{E3CF4B51-38E0-406C-92F3-D18A1127C00B}"/>
+  <autoFilter ref="B4:O4" xr:uid="{E3CF4B51-38E0-406C-92F3-D18A1127C00B}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>